<commit_message>
Admin leave management modify
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/OrangeHRM_TestData.xlsx
+++ b/src/test/resources/testdata/OrangeHRM_TestData.xlsx
@@ -1,27 +1,93 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{2D5C80F2-0501-43E0-97CB-AA7DC89561B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Leave Test data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <r>
+      <t>From</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>date</t>
+    </r>
+  </si>
+  <si>
+    <t>To date</t>
+  </si>
+  <si>
+    <t>Leave status</t>
+  </si>
+  <si>
+    <t>Leave type</t>
+  </si>
+  <si>
+    <t>Employee name</t>
+  </si>
+  <si>
+    <t>2026-31-12</t>
+  </si>
+  <si>
+    <t>Pending Approval</t>
+  </si>
+  <si>
+    <t>Ravi M B</t>
+  </si>
+  <si>
+    <t>2026-01-01</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -44,21 +110,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -96,7 +175,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -168,7 +247,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -341,10 +420,49 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
+    <col min="2" max="2" width="10.21875" customWidth="1"/>
+    <col min="3" max="3" width="14.77734375" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>